<commit_message>
feat: Enhance user import functionality and improve table filtering logic
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/public/assets/templates/template_user.xlsx
+++ b/public/assets/templates/template_user.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\kademangan\public\assets\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7CA6898-0308-416E-8F38-3DE39A3616FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11A8F5EF-8AB3-4946-8D9B-007D9BB8B622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{C540B8D7-40A2-45B0-835A-80841E5D2C9B}"/>
   </bookViews>
@@ -34,15 +34,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>nama_lengkap</t>
   </si>
   <si>
     <t>username</t>
-  </si>
-  <si>
-    <t>password</t>
   </si>
   <si>
     <t>id_level</t>
@@ -53,30 +50,12 @@
   <si>
     <t>jabatan_id</t>
   </si>
-  <si>
-    <t>(Contoh: Budi)</t>
-  </si>
-  <si>
-    <t>(Contoh: budi123)</t>
-  </si>
-  <si>
-    <t>(Contoh: rahasia123)</t>
-  </si>
-  <si>
-    <t>(Isi Angka)</t>
-  </si>
-  <si>
-    <t>(Opsional)</t>
-  </si>
-  <si>
-    <t>(Isi Angka/Kosong)</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -97,6 +76,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -106,7 +91,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -114,31 +99,17 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -455,48 +426,47 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA4FE568-50ED-4EB7-A747-B800E438D8D1}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:6" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" ht="28" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
     </row>
-    <row r="2" spans="1:6" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>11</v>
-      </c>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>